<commit_message>
Fix GDS units (um, not mm) and die grid quadrant convention
- GDS-X/GDS-Y are in micrometers, not millimeters. Convert to mm
  internally for plotting against die size (mm), and display the
  original um values in tooltips/detail list.
- die_X/die_Y are non-negative, first-quadrant indices, not a grid
  centered on (0,0). computeDieGrid still generates a symmetric grid
  internally (needed to test wafer-circle overlap) but now shifts the
  reported index by (maxI, maxJ) so die (0,0) is the grid's corner and
  the wafer center sits at (maxI, maxJ), auto-derived from wafer/die
  size.
- Regenerate sample_defects.csv/.xlsx to match: die indices shifted by
  +31/+31 (this wafer/die size's center), GDS values scaled x1000 to
  um. Verified all sample rows still land on valid wafer dies under
  the new convention.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-data/sample_defects.xlsx
+++ b/sample-data/sample_defects.xlsx
@@ -421,16 +421,16 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C2">
-        <v>0.5</v>
+        <v>500</v>
       </c>
       <c r="D2">
-        <v>0.3</v>
+        <v>300</v>
       </c>
       <c r="E2" t="str">
         <v>Particle</v>
@@ -441,16 +441,16 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C3">
-        <v>-1.2</v>
+        <v>-1200</v>
       </c>
       <c r="D3">
-        <v>0.9</v>
+        <v>900</v>
       </c>
       <c r="E3" t="str">
         <v>Scratch</v>
@@ -461,16 +461,16 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="D4">
-        <v>-1</v>
+        <v>-1000</v>
       </c>
       <c r="E4" t="str">
         <v>Particle</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -501,16 +501,16 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>-1</v>
+        <v>30</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C6">
-        <v>1.5</v>
+        <v>1500</v>
       </c>
       <c r="D6">
-        <v>1.5</v>
+        <v>1500</v>
       </c>
       <c r="E6" t="str">
         <v>Particle</v>
@@ -521,16 +521,16 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>-1</v>
+        <v>30</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>-1.5</v>
+        <v>-1500</v>
       </c>
       <c r="D7">
-        <v>-1.5</v>
+        <v>-1500</v>
       </c>
       <c r="E7" t="str">
         <v>Particle</v>
@@ -541,16 +541,16 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>-1</v>
+        <v>30</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C8">
-        <v>0.8</v>
+        <v>800</v>
       </c>
       <c r="D8">
-        <v>-0.6</v>
+        <v>-600</v>
       </c>
       <c r="E8" t="str">
         <v>Scratch</v>
@@ -561,16 +561,16 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="B9">
-        <v>-2</v>
+        <v>29</v>
       </c>
       <c r="C9">
-        <v>-0.4</v>
+        <v>-400</v>
       </c>
       <c r="D9">
-        <v>1.9</v>
+        <v>1900</v>
       </c>
       <c r="E9" t="str">
         <v>Bridge</v>
@@ -581,16 +581,16 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="B10">
-        <v>-2</v>
+        <v>29</v>
       </c>
       <c r="C10">
-        <v>1.9</v>
+        <v>1900</v>
       </c>
       <c r="D10">
-        <v>-0.4</v>
+        <v>-400</v>
       </c>
       <c r="E10" t="str">
         <v>Bridge</v>
@@ -601,16 +601,16 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="B11">
-        <v>-2</v>
+        <v>29</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
-        <v>-2</v>
+        <v>-2000</v>
       </c>
       <c r="E11" t="str">
         <v>Particle</v>
@@ -621,16 +621,16 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="B12">
-        <v>-3</v>
+        <v>28</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="E12" t="str">
         <v>Particle</v>
@@ -641,16 +641,16 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>-4</v>
+        <v>27</v>
       </c>
       <c r="B13">
-        <v>-2</v>
+        <v>29</v>
       </c>
       <c r="C13">
-        <v>-1.8</v>
+        <v>-1800</v>
       </c>
       <c r="D13">
-        <v>0.2</v>
+        <v>200</v>
       </c>
       <c r="E13" t="str">
         <v>Scratch</v>
@@ -661,16 +661,16 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C14">
-        <v>0.3</v>
+        <v>300</v>
       </c>
       <c r="D14">
-        <v>-1.7</v>
+        <v>-1700</v>
       </c>
       <c r="E14" t="str">
         <v>Void</v>
@@ -681,16 +681,16 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C15">
-        <v>-2</v>
+        <v>-2000</v>
       </c>
       <c r="D15">
-        <v>0.6</v>
+        <v>600</v>
       </c>
       <c r="E15" t="str">
         <v>Particle</v>
@@ -701,16 +701,16 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>-3</v>
+        <v>28</v>
       </c>
       <c r="B16">
-        <v>-4</v>
+        <v>27</v>
       </c>
       <c r="C16">
-        <v>0.9</v>
+        <v>900</v>
       </c>
       <c r="D16">
-        <v>0.9</v>
+        <v>900</v>
       </c>
       <c r="E16" t="str">
         <v>Particle</v>
@@ -721,16 +721,16 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>-3</v>
+        <v>28</v>
       </c>
       <c r="B17">
-        <v>-4</v>
+        <v>27</v>
       </c>
       <c r="C17">
-        <v>-0.9</v>
+        <v>-900</v>
       </c>
       <c r="D17">
-        <v>-0.9</v>
+        <v>-900</v>
       </c>
       <c r="E17" t="str">
         <v>Particle</v>
@@ -741,16 +741,16 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>-3</v>
+        <v>28</v>
       </c>
       <c r="B18">
-        <v>-4</v>
+        <v>27</v>
       </c>
       <c r="C18">
-        <v>1.4</v>
+        <v>1400</v>
       </c>
       <c r="D18">
-        <v>-1.4</v>
+        <v>-1400</v>
       </c>
       <c r="E18" t="str">
         <v>Particle</v>
@@ -761,16 +761,16 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>-3</v>
+        <v>28</v>
       </c>
       <c r="B19">
-        <v>-4</v>
+        <v>27</v>
       </c>
       <c r="C19">
-        <v>-1.4</v>
+        <v>-1400</v>
       </c>
       <c r="D19">
-        <v>1.4</v>
+        <v>1400</v>
       </c>
       <c r="E19" t="str">
         <v>Particle</v>
@@ -781,16 +781,16 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>-3</v>
+        <v>28</v>
       </c>
       <c r="B20">
-        <v>-4</v>
+        <v>27</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="E20" t="str">
         <v>Bridge</v>
@@ -801,13 +801,13 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>-3</v>
+        <v>28</v>
       </c>
       <c r="B21">
-        <v>-4</v>
+        <v>27</v>
       </c>
       <c r="C21">
-        <v>-2</v>
+        <v>-2000</v>
       </c>
       <c r="D21">
         <v>0</v>

</xml_diff>

<commit_message>
Add ECID/CQC-number hover support and a ruler on the die defect map
- Recognize an optional ECID column (aliases: ECID, CQC number, CQC
  ID, CQC) alongside the existing required columns. Wafer map hover
  now lists the die's ECID(s) next to its coordinate and defect
  count; die defect map hover/detail-list gets ECID as a dedicated
  field instead of being buried in the generic extra-columns dump.
- Add a ruler to the die defect map: tick marks with um labels along
  both axes, spaced at an auto-chosen "nice" interval (1/2/5 x 10^n)
  based on die size, so defect offsets can be read visually.
- Add a CQC number column (column A) to the sample CSV/XLSX, one ID
  per die, and verify the alias matching against it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-data/sample_defects.xlsx
+++ b/sample-data/sample_defects.xlsx
@@ -397,431 +397,494 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>CQC number</v>
+      </c>
+      <c r="B1" t="str">
         <v>die_X</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>die_Y</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>GDS-X</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>GDS-Y</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>defect_class</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>defect_size_um</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>31</v>
+      <c r="A2" t="str">
+        <v>CQC-100001</v>
       </c>
       <c r="B2">
         <v>31</v>
       </c>
       <c r="C2">
+        <v>31</v>
+      </c>
+      <c r="D2">
         <v>500</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>300</v>
       </c>
-      <c r="E2" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F2">
+      <c r="F2" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G2">
         <v>0.8</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>31</v>
+      <c r="A3" t="str">
+        <v>CQC-100001</v>
       </c>
       <c r="B3">
         <v>31</v>
       </c>
       <c r="C3">
+        <v>31</v>
+      </c>
+      <c r="D3">
         <v>-1200</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>900</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Scratch</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>1.4</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" t="str">
+        <v>CQC-100002</v>
+      </c>
+      <c r="B4">
         <v>32</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>31</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>2000</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>-1000</v>
       </c>
-      <c r="E4" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F4">
+      <c r="F4" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G4">
         <v>0.5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <v>32</v>
+      <c r="A5" t="str">
+        <v>CQC-100003</v>
       </c>
       <c r="B5">
         <v>32</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
         <v>Void</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>2.1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" t="str">
+        <v>CQC-100004</v>
+      </c>
+      <c r="B6">
         <v>30</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>32</v>
-      </c>
-      <c r="C6">
-        <v>1500</v>
       </c>
       <c r="D6">
         <v>1500</v>
       </c>
-      <c r="E6" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F6">
+      <c r="E6">
+        <v>1500</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G6">
         <v>0.6</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7">
+      <c r="A7" t="str">
+        <v>CQC-100004</v>
+      </c>
+      <c r="B7">
         <v>30</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>32</v>
-      </c>
-      <c r="C7">
-        <v>-1500</v>
       </c>
       <c r="D7">
         <v>-1500</v>
       </c>
-      <c r="E7" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F7">
+      <c r="E7">
+        <v>-1500</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G7">
         <v>0.7</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8">
+      <c r="A8" t="str">
+        <v>CQC-100004</v>
+      </c>
+      <c r="B8">
         <v>30</v>
       </c>
-      <c r="B8">
+      <c r="C8">
         <v>32</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>800</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>-600</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>Scratch</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9">
+      <c r="A9" t="str">
+        <v>CQC-100005</v>
+      </c>
+      <c r="B9">
         <v>33</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>29</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>-400</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>1900</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>Bridge</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>3.2</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10">
+      <c r="A10" t="str">
+        <v>CQC-100005</v>
+      </c>
+      <c r="B10">
         <v>33</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>29</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>1900</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>-400</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>Bridge</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>2.8</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11">
+      <c r="A11" t="str">
+        <v>CQC-100005</v>
+      </c>
+      <c r="B11">
         <v>33</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>29</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>0</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>-2000</v>
       </c>
-      <c r="E11" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F11">
+      <c r="F11" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G11">
         <v>0.4</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12">
+      <c r="A12" t="str">
+        <v>CQC-100006</v>
+      </c>
+      <c r="B12">
         <v>31</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>28</v>
-      </c>
-      <c r="C12">
-        <v>1000</v>
       </c>
       <c r="D12">
         <v>1000</v>
       </c>
-      <c r="E12" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F12">
+      <c r="E12">
+        <v>1000</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G12">
         <v>0.5</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13">
+      <c r="A13" t="str">
+        <v>CQC-100007</v>
+      </c>
+      <c r="B13">
         <v>27</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>29</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>-1800</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>200</v>
       </c>
-      <c r="E13" t="str">
+      <c r="F13" t="str">
         <v>Scratch</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>1.1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14">
+      <c r="A14" t="str">
+        <v>CQC-100008</v>
+      </c>
+      <c r="B14">
         <v>36</v>
       </c>
-      <c r="B14">
+      <c r="C14">
         <v>32</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <v>300</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>-1700</v>
       </c>
-      <c r="E14" t="str">
+      <c r="F14" t="str">
         <v>Void</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>1.9</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15">
+      <c r="A15" t="str">
+        <v>CQC-100008</v>
+      </c>
+      <c r="B15">
         <v>36</v>
       </c>
-      <c r="B15">
+      <c r="C15">
         <v>32</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>-2000</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>600</v>
       </c>
-      <c r="E15" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F15">
+      <c r="F15" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G15">
         <v>0.6</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16">
+      <c r="A16" t="str">
+        <v>CQC-100009</v>
+      </c>
+      <c r="B16">
         <v>28</v>
       </c>
-      <c r="B16">
+      <c r="C16">
         <v>27</v>
-      </c>
-      <c r="C16">
-        <v>900</v>
       </c>
       <c r="D16">
         <v>900</v>
       </c>
-      <c r="E16" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F16">
+      <c r="E16">
+        <v>900</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G16">
         <v>0.5</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17">
+      <c r="A17" t="str">
+        <v>CQC-100009</v>
+      </c>
+      <c r="B17">
         <v>28</v>
       </c>
-      <c r="B17">
+      <c r="C17">
         <v>27</v>
-      </c>
-      <c r="C17">
-        <v>-900</v>
       </c>
       <c r="D17">
         <v>-900</v>
       </c>
-      <c r="E17" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F17">
+      <c r="E17">
+        <v>-900</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G17">
         <v>0.5</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18">
+      <c r="A18" t="str">
+        <v>CQC-100009</v>
+      </c>
+      <c r="B18">
         <v>28</v>
       </c>
-      <c r="B18">
+      <c r="C18">
         <v>27</v>
       </c>
-      <c r="C18">
+      <c r="D18">
         <v>1400</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>-1400</v>
       </c>
-      <c r="E18" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F18">
+      <c r="F18" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G18">
         <v>0.5</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19">
+      <c r="A19" t="str">
+        <v>CQC-100009</v>
+      </c>
+      <c r="B19">
         <v>28</v>
       </c>
-      <c r="B19">
+      <c r="C19">
         <v>27</v>
       </c>
-      <c r="C19">
+      <c r="D19">
         <v>-1400</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>1400</v>
       </c>
-      <c r="E19" t="str">
-        <v>Particle</v>
-      </c>
-      <c r="F19">
+      <c r="F19" t="str">
+        <v>Particle</v>
+      </c>
+      <c r="G19">
         <v>0.5</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20">
+      <c r="A20" t="str">
+        <v>CQC-100009</v>
+      </c>
+      <c r="B20">
         <v>28</v>
       </c>
-      <c r="B20">
+      <c r="C20">
         <v>27</v>
       </c>
-      <c r="C20">
+      <c r="D20">
         <v>0</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>2000</v>
       </c>
-      <c r="E20" t="str">
+      <c r="F20" t="str">
         <v>Bridge</v>
       </c>
-      <c r="F20">
+      <c r="G20">
         <v>4</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21">
+      <c r="A21" t="str">
+        <v>CQC-100009</v>
+      </c>
+      <c r="B21">
         <v>28</v>
       </c>
-      <c r="B21">
+      <c r="C21">
         <v>27</v>
       </c>
-      <c r="C21">
+      <c r="D21">
         <v>-2000</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>0</v>
       </c>
-      <c r="E21" t="str">
+      <c r="F21" t="str">
         <v>Bridge</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>3.6</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>